<commit_message>
Recommit without large pptx
</commit_message>
<xml_diff>
--- a/data/transcripts/Codes.xlsx
+++ b/data/transcripts/Codes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JoeWe\IndProj\Project\data\transcripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F786FA8-CA6D-495E-82F1-9ECDDDE33AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E208C2DE-F465-43CD-A16D-83488D693B82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{AC90B9A7-A62A-404B-BF46-87E4220995B1}"/>
   </bookViews>
@@ -264,11 +264,6 @@
     <t>For visualisation, I think the closer you get to target, maybe swap modes like I said, like the radar.</t>
   </si>
   <si>
-    <t>Filter noise out and like so.
-So if there's like an ambient sound going on, let's say like a a washing machine or like a fan going on.
-It will know how to filter it out.</t>
-  </si>
-  <si>
     <t>Uh, and then I think the lights were pretty useful for like when you actually got right to the sound because.
 Well, the other ones they they spun out like a compass, but yeah, I guess you kind of knew which way exactly to look because one side would one side would go off.</t>
   </si>
@@ -447,6 +442,11 @@
   <si>
     <t xml:space="preserve"> Participant:  Or in a working environment that perhaps has too many things for somebody to...
  Participant:  keep track of. So like a, you know, the system takes care of is an extra help with awareness. Maybe you're focused on what you're doing and you need an extra help to say, oh, watch your left, watch your right, or look left, look right.</t>
+  </si>
+  <si>
+    <t>Have it where I can like, Filter noise out and like so.
+So if there's like an ambient sound going on, let's say like a a washing machine or like a fan going on.
+It will know how to filter it out.</t>
   </si>
 </sst>
 </file>
@@ -878,7 +878,7 @@
     </row>
     <row r="5" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5">
         <v>5</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="6" spans="1:4" ht="57" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>7</v>
@@ -922,7 +922,7 @@
     </row>
     <row r="9" spans="1:4" ht="156.75" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B9">
         <v>5</v>
@@ -933,7 +933,7 @@
     </row>
     <row r="10" spans="1:4" ht="199.5" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10">
         <v>7</v>
@@ -944,7 +944,7 @@
     </row>
     <row r="11" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11">
         <v>9</v>
@@ -955,7 +955,7 @@
     </row>
     <row r="12" spans="1:4" ht="128.25" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B12">
         <v>9</v>
@@ -977,7 +977,7 @@
     </row>
     <row r="14" spans="1:4" ht="299.25" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B14">
         <v>5</v>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="18" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18">
         <v>5</v>
@@ -1032,7 +1032,7 @@
     </row>
     <row r="19" spans="1:3" ht="57" x14ac:dyDescent="0.45">
       <c r="A19" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B19">
         <v>7</v>
@@ -1043,7 +1043,7 @@
     </row>
     <row r="20" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A20" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B20">
         <v>5</v>
@@ -1054,7 +1054,7 @@
     </row>
     <row r="21" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B21">
         <v>7</v>
@@ -1065,7 +1065,7 @@
     </row>
     <row r="22" spans="1:3" ht="57" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22">
         <v>8</v>
@@ -1076,7 +1076,7 @@
     </row>
     <row r="23" spans="1:3" ht="57" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B23">
         <v>9</v>
@@ -1120,7 +1120,7 @@
     </row>
     <row r="27" spans="1:3" ht="142.5" x14ac:dyDescent="0.45">
       <c r="A27" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B27">
         <v>5</v>
@@ -1131,7 +1131,7 @@
     </row>
     <row r="28" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A28" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B28">
         <v>9</v>
@@ -1142,7 +1142,7 @@
     </row>
     <row r="29" spans="1:3" ht="114" x14ac:dyDescent="0.45">
       <c r="A29" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B29">
         <v>9</v>
@@ -1153,7 +1153,7 @@
     </row>
     <row r="30" spans="1:3" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A30" s="1" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="B30">
         <v>4</v>
@@ -1164,7 +1164,7 @@
     </row>
     <row r="31" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A31" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B31">
         <v>6</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="33" spans="1:3" ht="171" x14ac:dyDescent="0.45">
       <c r="A33" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B33">
         <v>6</v>
@@ -1197,7 +1197,7 @@
     </row>
     <row r="34" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A34" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B34">
         <v>9</v>
@@ -1208,7 +1208,7 @@
     </row>
     <row r="35" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A35" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B35">
         <v>9</v>
@@ -1219,7 +1219,7 @@
     </row>
     <row r="36" spans="1:3" ht="57" x14ac:dyDescent="0.45">
       <c r="A36" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B36">
         <v>9</v>
@@ -1329,7 +1329,7 @@
     </row>
     <row r="46" spans="1:3" ht="171" x14ac:dyDescent="0.45">
       <c r="A46" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B46">
         <v>5</v>
@@ -1340,7 +1340,7 @@
     </row>
     <row r="47" spans="1:3" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A47" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B47">
         <v>8</v>
@@ -1351,7 +1351,7 @@
     </row>
     <row r="48" spans="1:3" ht="342" x14ac:dyDescent="0.45">
       <c r="A48" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B48">
         <v>8</v>
@@ -1362,7 +1362,7 @@
     </row>
     <row r="49" spans="1:3" ht="57" x14ac:dyDescent="0.45">
       <c r="A49" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B49">
         <v>9</v>
@@ -1428,7 +1428,7 @@
     </row>
     <row r="55" spans="1:3" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A55" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B55">
         <v>6</v>
@@ -1439,7 +1439,7 @@
     </row>
     <row r="56" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A56" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B56">
         <v>8</v>
@@ -1480,7 +1480,7 @@
     </row>
     <row r="60" spans="1:3" ht="370.5" x14ac:dyDescent="0.45">
       <c r="A60" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B60">
         <v>5</v>
@@ -1491,7 +1491,7 @@
     </row>
     <row r="61" spans="1:3" ht="114" x14ac:dyDescent="0.45">
       <c r="A61" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B61">
         <v>9</v>
@@ -1502,7 +1502,7 @@
     </row>
     <row r="62" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A62" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B62">
         <v>9</v>
@@ -1568,7 +1568,7 @@
     </row>
     <row r="68" spans="1:3" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A68" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B68">
         <v>5</v>
@@ -1590,7 +1590,7 @@
     </row>
     <row r="70" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A70" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B70">
         <v>5</v>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="71" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A71" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B71">
         <v>5</v>
@@ -1645,7 +1645,7 @@
     </row>
     <row r="75" spans="1:3" ht="114" x14ac:dyDescent="0.45">
       <c r="A75" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B75">
         <v>5</v>
@@ -1656,7 +1656,7 @@
     </row>
     <row r="76" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A76" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B76">
         <v>5</v>
@@ -1667,7 +1667,7 @@
     </row>
     <row r="77" spans="1:3" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A77" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B77">
         <v>6</v>
@@ -1678,7 +1678,7 @@
     </row>
     <row r="78" spans="1:3" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A78" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B78">
         <v>7</v>
@@ -1689,7 +1689,7 @@
     </row>
     <row r="79" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A79" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B79">
         <v>9</v>
@@ -1711,7 +1711,7 @@
     </row>
     <row r="81" spans="1:3" ht="171" x14ac:dyDescent="0.45">
       <c r="A81" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B81">
         <v>5</v>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="82" spans="1:3" ht="171" x14ac:dyDescent="0.45">
       <c r="A82" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B82">
         <v>5</v>
@@ -1733,7 +1733,7 @@
     </row>
     <row r="83" spans="1:3" ht="171" x14ac:dyDescent="0.45">
       <c r="A83" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B83">
         <v>8</v>

</xml_diff>